<commit_message>
oh god quick add it all
</commit_message>
<xml_diff>
--- a/The Report/Requirements specification.xlsx
+++ b/The Report/Requirements specification.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kidic\Documents\Computer Science\Project Work\The Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{363DEB3D-2A72-4318-97A9-8BE3B03AD2F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F124A37-72C9-4BB9-92B1-923C9D661A41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="195">
   <si>
     <t>Requirement</t>
   </si>
@@ -119,9 +119,6 @@
     <t>Amounts Tracker</t>
   </si>
   <si>
-    <t>Expiration Detailer</t>
-  </si>
-  <si>
     <t>Taste Tracker</t>
   </si>
   <si>
@@ -228,9 +225,6 @@
   </si>
   <si>
     <t>https://github.com/JessHorserage/Marvellous-Meal-Maker/issues/12</t>
-  </si>
-  <si>
-    <t>https://github.com/JessHorserage/Marvellous-Meal-Maker/issues/13</t>
   </si>
   <si>
     <t>https://github.com/JessHorserage/Marvellous-Meal-Maker/issues/14</t>
@@ -437,16 +431,6 @@
 Tied into specific items</t>
   </si>
   <si>
-    <t>Expiration methodologies and timings for items</t>
-  </si>
-  <si>
-    <t>Items need to be good for certain amounts of time in meals and for further usage, so knowing expirations helps a lot</t>
-  </si>
-  <si>
-    <t>Expiration dates
-Expiration methods</t>
-  </si>
-  <si>
     <t>Allocates different tastes to items</t>
   </si>
   <si>
@@ -666,6 +650,9 @@
   </si>
   <si>
     <t>Specific hard to obtain ingredients or allergens in recipes might be able to be bodged from a variety of specific items into bodged products</t>
+  </si>
+  <si>
+    <t>Now contains the previous expiration tracker</t>
   </si>
 </sst>
 </file>
@@ -774,8 +761,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C60201B-D876-4109-8647-FE7C1079C08C}" name="Table1" displayName="Table1" ref="B2:I39" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="B2:I39" xr:uid="{1C60201B-D876-4109-8647-FE7C1079C08C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1C60201B-D876-4109-8647-FE7C1079C08C}" name="Table1" displayName="Table1" ref="B2:I38" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="B2:I38" xr:uid="{1C60201B-D876-4109-8647-FE7C1079C08C}"/>
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{61333736-D8AE-4E92-8083-E0CA1447312A}" name="Requirement" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{3BFEB35C-ED06-4F45-ABB0-1959FF28BE4A}" name="Subrequirement" dataDxfId="6"/>
@@ -1097,12 +1084,12 @@
         <v>6</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="3" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="1">
         <v>1</v>
@@ -1111,13 +1098,13 @@
         <v>15</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K3" s="1" t="s">
         <v>9</v>
@@ -1137,19 +1124,19 @@
         <v>16</v>
       </c>
       <c r="E4" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="H4" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="F4" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>93</v>
-      </c>
       <c r="I4" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="K4" s="1" t="s">
         <v>5</v>
@@ -1160,7 +1147,7 @@
     </row>
     <row r="5" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" s="1">
         <v>1.2</v>
@@ -1169,19 +1156,19 @@
         <v>17</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F5" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I5" s="2" t="s">
         <v>51</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>52</v>
       </c>
       <c r="K5" s="1" t="s">
         <v>13</v>
@@ -1192,7 +1179,7 @@
     </row>
     <row r="6" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C6" s="1">
         <v>1.3</v>
@@ -1201,19 +1188,22 @@
         <v>18</v>
       </c>
       <c r="E6" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H6" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>99</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>194</v>
       </c>
       <c r="K6" s="1" t="s">
         <v>14</v>
@@ -1224,7 +1214,7 @@
     </row>
     <row r="7" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C7" s="1">
         <v>1.4</v>
@@ -1233,30 +1223,30 @@
         <v>19</v>
       </c>
       <c r="E7" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="H7" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="F7" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>102</v>
-      </c>
       <c r="I7" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="K7" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L7" s="1" t="s">
         <v>49</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="8" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C8" s="1">
         <v>1.5</v>
@@ -1265,24 +1255,24 @@
         <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="H8" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="F8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>105</v>
-      </c>
       <c r="I8" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C9" s="1">
         <v>1.6</v>
@@ -1291,22 +1281,22 @@
         <v>21</v>
       </c>
       <c r="E9" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="H9" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="F9" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>108</v>
-      </c>
       <c r="I9" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -1320,24 +1310,24 @@
         <v>22</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C11" s="1">
         <v>1.8</v>
@@ -1346,19 +1336,19 @@
         <v>23</v>
       </c>
       <c r="E11" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="H11" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="H11" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="I11" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -1372,19 +1362,19 @@
         <v>24</v>
       </c>
       <c r="E12" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="H12" s="1" t="s">
         <v>114</v>
       </c>
-      <c r="F12" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>116</v>
-      </c>
       <c r="I12" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
@@ -1398,30 +1388,30 @@
         <v>25</v>
       </c>
       <c r="E13" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="F13" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="K13" s="1" t="s">
         <v>121</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="J13" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="14" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C14" s="1">
         <v>1.1100000000000001</v>
@@ -1430,24 +1420,24 @@
         <v>26</v>
       </c>
       <c r="E14" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="F14" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>128</v>
-      </c>
       <c r="I14" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="C15" s="1">
         <v>1.1200000000000001</v>
@@ -1456,123 +1446,123 @@
         <v>27</v>
       </c>
       <c r="E15" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="H15" s="1" t="s">
         <v>129</v>
       </c>
-      <c r="F15" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G15" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="H15" s="1" t="s">
-        <v>131</v>
-      </c>
       <c r="I15" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="16" spans="2:12" ht="57.6" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C16" s="1">
-        <v>1.1299999999999999</v>
+        <v>2</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>28</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I16" s="2" t="s">
-        <v>65</v>
+        <v>46</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>53</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="17" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="C17" s="1">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>29</v>
       </c>
       <c r="E17" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="H17" s="1" t="s">
         <v>138</v>
       </c>
-      <c r="F17" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="I17" s="1" t="s">
-        <v>54</v>
+      <c r="I17" s="2" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="18" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C18" s="1">
-        <v>2.1</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>30</v>
       </c>
       <c r="E18" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="H18" s="1" t="s">
         <v>141</v>
       </c>
-      <c r="F18" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G18" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>143</v>
-      </c>
       <c r="I18" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="19" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
-        <v>49</v>
+        <v>13</v>
       </c>
       <c r="C19" s="1">
-        <v>2.2000000000000002</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>31</v>
       </c>
       <c r="E19" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>144</v>
       </c>
-      <c r="F19" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G19" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>146</v>
-      </c>
       <c r="I19" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
@@ -1580,59 +1570,59 @@
         <v>13</v>
       </c>
       <c r="C20" s="1">
-        <v>2.2999999999999998</v>
+        <v>2.4</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>32</v>
       </c>
       <c r="E20" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G20" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="F20" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G20" s="1" t="s">
+      <c r="H20" s="1" t="s">
         <v>148</v>
       </c>
-      <c r="H20" s="1" t="s">
-        <v>149</v>
-      </c>
       <c r="I20" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="21" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
-        <v>13</v>
+        <v>48</v>
       </c>
       <c r="C21" s="1">
-        <v>2.4</v>
+        <v>2.5</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>33</v>
       </c>
       <c r="E21" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="H21" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="F21" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G21" s="1" t="s">
-        <v>152</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>153</v>
-      </c>
       <c r="I21" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="22" spans="2:9" ht="43.2" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C22" s="1">
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>34</v>
@@ -1641,200 +1631,200 @@
         <v>151</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="I22" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="23" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C23" s="1">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>35</v>
+        <v>70</v>
       </c>
       <c r="E23" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G23" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G23" s="1" t="s">
+      <c r="H23" s="1" t="s">
         <v>157</v>
       </c>
-      <c r="H23" s="1" t="s">
-        <v>158</v>
-      </c>
       <c r="I23" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="24" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C24" s="1">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="D24" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" ht="72" x14ac:dyDescent="0.3">
+      <c r="B25" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C25" s="1">
+        <v>2.9</v>
+      </c>
+      <c r="D25" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="E24" s="1" t="s">
-        <v>159</v>
-      </c>
-      <c r="F24" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G24" s="1" t="s">
-        <v>161</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="25" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B25" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C25" s="1">
-        <v>2.8</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>160</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G25" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="H25" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="H25" s="1" t="s">
-        <v>164</v>
-      </c>
       <c r="I25" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="26" spans="2:9" ht="72" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C26" s="1">
-        <v>2.9</v>
+        <v>2.101</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>167</v>
+        <v>193</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="27" spans="2:9" ht="72" x14ac:dyDescent="0.3">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C27" s="1">
-        <v>2.101</v>
+        <v>3</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>75</v>
+        <v>35</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>166</v>
+        <v>134</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="I27" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="28" spans="2:9" ht="28.8" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B28" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C28" s="1">
-        <v>3</v>
+        <v>3.1</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>36</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>139</v>
+        <v>165</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I28" s="1" t="s">
-        <v>54</v>
+        <v>50</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B29" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C29" s="1">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>37</v>
       </c>
       <c r="E29" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H29" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="F29" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G29" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="H29" s="1" t="s">
-        <v>172</v>
-      </c>
       <c r="I29" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="30" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C30" s="1">
-        <v>3.2</v>
+        <v>3.3</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>38</v>
@@ -1843,286 +1833,260 @@
         <v>173</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="31" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" x14ac:dyDescent="0.3">
       <c r="B31" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C31" s="1">
-        <v>3.3</v>
+        <v>3</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>178</v>
+        <v>135</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>82</v>
+        <v>50</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>53</v>
       </c>
     </row>
     <row r="32" spans="2:9" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C32" s="1">
-        <v>3</v>
+        <v>3.4</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>140</v>
+        <v>174</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="I32" s="1" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="33" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
+        <v>50</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="72" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C33" s="1">
-        <v>3.4</v>
+        <v>3.5</v>
       </c>
       <c r="D33" s="1" t="s">
         <v>40</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G33" s="1" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="H33" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="2:9" ht="72" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C34" s="1">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="D34" s="1" t="s">
         <v>41</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G34" s="1" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H34" s="1" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="35" spans="2:9" ht="72" x14ac:dyDescent="0.3">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B35" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C35" s="1">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="D35" s="1" t="s">
         <v>42</v>
       </c>
       <c r="E35" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="H35" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="F35" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>185</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>186</v>
-      </c>
       <c r="I35" s="2" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="36" spans="2:9" ht="86.4" x14ac:dyDescent="0.3">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B36" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C36" s="1">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="D36" s="1" t="s">
         <v>43</v>
       </c>
       <c r="E36" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="H36" s="1" t="s">
         <v>188</v>
       </c>
-      <c r="F36" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>189</v>
-      </c>
       <c r="I36" s="2" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="37" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" ht="72" x14ac:dyDescent="0.3">
       <c r="B37" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C37" s="1">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="D37" s="1" t="s">
         <v>44</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>190</v>
       </c>
-      <c r="F37" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>192</v>
-      </c>
       <c r="H37" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="38" spans="2:9" ht="72" x14ac:dyDescent="0.3">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B38" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C38" s="1">
-        <v>3.9</v>
+        <v>1.1299999999999999</v>
       </c>
       <c r="D38" s="1" t="s">
         <v>45</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>194</v>
+        <v>130</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G38" s="1" t="s">
-        <v>195</v>
+        <v>131</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>196</v>
+        <v>132</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="39" spans="2:9" ht="57.6" x14ac:dyDescent="0.3">
-      <c r="B39" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C39" s="1">
-        <v>1.1399999999999999</v>
-      </c>
-      <c r="D39" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="F39" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="H39" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>89</v>
-      </c>
-    </row>
+        <v>87</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>
-    <hyperlink ref="I19" r:id="rId1" xr:uid="{A22FC6E8-013D-4B9C-888B-6DEB66BC0BBD}"/>
-    <hyperlink ref="I18" r:id="rId2" xr:uid="{7C396296-C385-4A00-99E1-988F34796E1E}"/>
-    <hyperlink ref="I16" r:id="rId3" xr:uid="{76D81C8E-FB21-48C0-9F0B-93BC9FA5FA75}"/>
-    <hyperlink ref="I15" r:id="rId4" xr:uid="{A0067A10-2FBD-4665-B9A8-9F882E7F7B5E}"/>
-    <hyperlink ref="I14" r:id="rId5" xr:uid="{B4CD3B35-5559-43F7-A63F-A73946B25C09}"/>
-    <hyperlink ref="I13" r:id="rId6" xr:uid="{C8ABCD4A-CD74-4563-B37C-B6E3BADAED14}"/>
-    <hyperlink ref="I12" r:id="rId7" xr:uid="{14C15A46-F60D-4C6C-9780-68099ABDBDBE}"/>
-    <hyperlink ref="I11" r:id="rId8" xr:uid="{9180ABAD-38CF-4BD5-B15E-087B315799D4}"/>
-    <hyperlink ref="I10" r:id="rId9" xr:uid="{C93B0FDF-9812-4DBA-98A5-57B245D68060}"/>
-    <hyperlink ref="I9" r:id="rId10" xr:uid="{192DEBE5-436F-4648-BD53-254A2FD5559D}"/>
-    <hyperlink ref="I8" r:id="rId11" xr:uid="{8741CBAE-DA1E-4AB2-89D0-15E13AF26114}"/>
-    <hyperlink ref="I7" r:id="rId12" xr:uid="{31AE8EC8-0886-4AE6-89A9-146FF6280707}"/>
-    <hyperlink ref="I6" r:id="rId13" xr:uid="{85D839C6-4686-4DBE-B3C1-93828D05BEDC}"/>
-    <hyperlink ref="I5" r:id="rId14" xr:uid="{E1658E24-0100-45FF-B91E-6530B50A13E2}"/>
-    <hyperlink ref="I4" r:id="rId15" xr:uid="{FB7FB13B-DAE9-4C5A-A4DE-EE374878EC92}"/>
-    <hyperlink ref="I20" r:id="rId16" xr:uid="{1C280FCF-5DC4-4792-8AC5-AE3CE8585DC6}"/>
-    <hyperlink ref="I21" r:id="rId17" xr:uid="{C514906A-02C9-43EA-BEE8-30E741748FD0}"/>
-    <hyperlink ref="I22" r:id="rId18" xr:uid="{DB44C35E-F0B0-42F8-A92B-4C36CADAB8ED}"/>
-    <hyperlink ref="I23" r:id="rId19" xr:uid="{B806D4F2-CDA0-47E0-9AE2-FC9F3918EB5A}"/>
-    <hyperlink ref="I24" r:id="rId20" xr:uid="{50239B50-B1BF-4833-B28B-545339B02172}"/>
-    <hyperlink ref="I25" r:id="rId21" xr:uid="{7FE2DFCA-6167-4F14-8F20-37CF0E1CAE10}"/>
-    <hyperlink ref="I27" r:id="rId22" xr:uid="{BB1F3120-FDCE-44A7-A68E-FE1A2F19B08A}"/>
-    <hyperlink ref="I26" r:id="rId23" xr:uid="{5A54E90B-0719-4091-8771-E641A56EF2B0}"/>
-    <hyperlink ref="I29" r:id="rId24" xr:uid="{6B646C5C-3904-4E32-8163-2AB83854CE47}"/>
-    <hyperlink ref="I39" r:id="rId25" xr:uid="{25F7B40E-9B47-4B3B-94A9-8C6A350B7958}"/>
-    <hyperlink ref="I38" r:id="rId26" xr:uid="{B0B53DF3-B6C8-42B3-B464-730198107A65}"/>
-    <hyperlink ref="I37" r:id="rId27" xr:uid="{99837656-CD4A-4C54-AECC-E07BA118DB08}"/>
-    <hyperlink ref="I36" r:id="rId28" xr:uid="{2688C20B-5A64-4ED9-82C8-81719A512998}"/>
-    <hyperlink ref="I35" r:id="rId29" xr:uid="{F105F2F7-05F0-4C22-95B7-206D2C61766B}"/>
-    <hyperlink ref="I34" r:id="rId30" xr:uid="{78811BCE-8910-4021-9F8A-F2CF05DCAC11}"/>
-    <hyperlink ref="I33" r:id="rId31" xr:uid="{8768ECC4-9661-455C-8301-5D4590E28B8B}"/>
-    <hyperlink ref="I31" r:id="rId32" xr:uid="{BB916ACE-4178-4366-8C88-91BFE05C4912}"/>
-    <hyperlink ref="I30" r:id="rId33" xr:uid="{CE7AD33D-23CB-42A0-A0A4-F16C2CAE0446}"/>
+    <hyperlink ref="I18" r:id="rId1" xr:uid="{A22FC6E8-013D-4B9C-888B-6DEB66BC0BBD}"/>
+    <hyperlink ref="I17" r:id="rId2" xr:uid="{7C396296-C385-4A00-99E1-988F34796E1E}"/>
+    <hyperlink ref="I15" r:id="rId3" xr:uid="{76D81C8E-FB21-48C0-9F0B-93BC9FA5FA75}"/>
+    <hyperlink ref="I14" r:id="rId4" xr:uid="{B4CD3B35-5559-43F7-A63F-A73946B25C09}"/>
+    <hyperlink ref="I13" r:id="rId5" xr:uid="{C8ABCD4A-CD74-4563-B37C-B6E3BADAED14}"/>
+    <hyperlink ref="I12" r:id="rId6" xr:uid="{14C15A46-F60D-4C6C-9780-68099ABDBDBE}"/>
+    <hyperlink ref="I11" r:id="rId7" xr:uid="{9180ABAD-38CF-4BD5-B15E-087B315799D4}"/>
+    <hyperlink ref="I10" r:id="rId8" xr:uid="{C93B0FDF-9812-4DBA-98A5-57B245D68060}"/>
+    <hyperlink ref="I9" r:id="rId9" xr:uid="{192DEBE5-436F-4648-BD53-254A2FD5559D}"/>
+    <hyperlink ref="I8" r:id="rId10" xr:uid="{8741CBAE-DA1E-4AB2-89D0-15E13AF26114}"/>
+    <hyperlink ref="I7" r:id="rId11" xr:uid="{31AE8EC8-0886-4AE6-89A9-146FF6280707}"/>
+    <hyperlink ref="I6" r:id="rId12" xr:uid="{85D839C6-4686-4DBE-B3C1-93828D05BEDC}"/>
+    <hyperlink ref="I5" r:id="rId13" xr:uid="{E1658E24-0100-45FF-B91E-6530B50A13E2}"/>
+    <hyperlink ref="I4" r:id="rId14" xr:uid="{FB7FB13B-DAE9-4C5A-A4DE-EE374878EC92}"/>
+    <hyperlink ref="I19" r:id="rId15" xr:uid="{1C280FCF-5DC4-4792-8AC5-AE3CE8585DC6}"/>
+    <hyperlink ref="I20" r:id="rId16" xr:uid="{C514906A-02C9-43EA-BEE8-30E741748FD0}"/>
+    <hyperlink ref="I21" r:id="rId17" xr:uid="{DB44C35E-F0B0-42F8-A92B-4C36CADAB8ED}"/>
+    <hyperlink ref="I22" r:id="rId18" xr:uid="{B806D4F2-CDA0-47E0-9AE2-FC9F3918EB5A}"/>
+    <hyperlink ref="I23" r:id="rId19" xr:uid="{50239B50-B1BF-4833-B28B-545339B02172}"/>
+    <hyperlink ref="I24" r:id="rId20" xr:uid="{7FE2DFCA-6167-4F14-8F20-37CF0E1CAE10}"/>
+    <hyperlink ref="I26" r:id="rId21" xr:uid="{BB1F3120-FDCE-44A7-A68E-FE1A2F19B08A}"/>
+    <hyperlink ref="I25" r:id="rId22" xr:uid="{5A54E90B-0719-4091-8771-E641A56EF2B0}"/>
+    <hyperlink ref="I28" r:id="rId23" xr:uid="{6B646C5C-3904-4E32-8163-2AB83854CE47}"/>
+    <hyperlink ref="I38" r:id="rId24" xr:uid="{25F7B40E-9B47-4B3B-94A9-8C6A350B7958}"/>
+    <hyperlink ref="I37" r:id="rId25" xr:uid="{B0B53DF3-B6C8-42B3-B464-730198107A65}"/>
+    <hyperlink ref="I36" r:id="rId26" xr:uid="{99837656-CD4A-4C54-AECC-E07BA118DB08}"/>
+    <hyperlink ref="I35" r:id="rId27" xr:uid="{2688C20B-5A64-4ED9-82C8-81719A512998}"/>
+    <hyperlink ref="I34" r:id="rId28" xr:uid="{F105F2F7-05F0-4C22-95B7-206D2C61766B}"/>
+    <hyperlink ref="I33" r:id="rId29" xr:uid="{78811BCE-8910-4021-9F8A-F2CF05DCAC11}"/>
+    <hyperlink ref="I32" r:id="rId30" xr:uid="{8768ECC4-9661-455C-8301-5D4590E28B8B}"/>
+    <hyperlink ref="I30" r:id="rId31" xr:uid="{BB916ACE-4178-4366-8C88-91BFE05C4912}"/>
+    <hyperlink ref="I29" r:id="rId32" xr:uid="{CE7AD33D-23CB-42A0-A0A4-F16C2CAE0446}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId34"/>
+    <tablePart r:id="rId33"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
todays dump from the master
</commit_message>
<xml_diff>
--- a/The Report/Requirements specification.xlsx
+++ b/The Report/Requirements specification.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kidic\Documents\Computer Science\Project Work\The Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Marvellous-Meal-Maker\The Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5334BE-6B02-413A-9E75-F3264ADE844E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D836034-176A-46FE-BB7A-26FAACC66CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="213">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="220">
   <si>
     <t>Requirement</t>
   </si>
@@ -706,7 +706,28 @@
     <t>ProductStorage, location stored as str times stored as int, shared with 1.3 AllocateProductStorage AllocateProductTimes</t>
   </si>
   <si>
-    <t xml:space="preserve">MethodsMethods, allocate if methods can be intermediary with a bool allocate the end result of an intermediary as its own separate but the same item registry, </t>
+    <t>MethodsMethods, allocate if methods can be intermediary with a bool allocate the end result of an intermediary as its own separate but the same item registry, AllocateIntermediary RemoveIntermediary LinkIntermediaryWithItem RemoveLinkIntermediaryWithItem</t>
+  </si>
+  <si>
+    <t>MethodCuisine, declarations of method cuisines as a str, DeclareCuisine DeleteCuisine AllocateCuisine RemoveCuisine ShowAllProductsCuisines ShowAllCuisinesProducts</t>
+  </si>
+  <si>
+    <t>Repeat from on high</t>
+  </si>
+  <si>
+    <t>MethodsAppend, the rest of this section</t>
+  </si>
+  <si>
+    <t>MethodsSetUp, set up time in minutes as int, SetMethodSetUp</t>
+  </si>
+  <si>
+    <t>MethodsCookUp, set up time in minutes as int, SetMethodCookUp</t>
+  </si>
+  <si>
+    <t>MethodVariant, items that can be changed are noted in their entry New recipe name stored as string if there is one Int for the amount of variants a thing has, DeclareMethodVariant ChangeMethodsVariants RemoveMethodVariant ListMethodVariants</t>
+  </si>
+  <si>
+    <t>MethodBodge, items that are bodging for something else are noted in the pantry and what they become in the pantry, DeclareMethodBodge ChangeMethodBodge RemoveMethodBodge ListMethodsVariants</t>
   </si>
 </sst>
 </file>
@@ -1099,24 +1120,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:M39"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="1"/>
-    <col min="2" max="2" width="14.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" style="1"/>
+    <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.6640625" style="1" customWidth="1"/>
-    <col min="8" max="8" width="24.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="49.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="47.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5546875" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="31.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.7109375" style="1" customWidth="1"/>
+    <col min="8" max="8" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="49.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="47.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5703125" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.85546875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1148,7 +1169,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:13" ht="45" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
         <v>48</v>
       </c>
@@ -1177,7 +1198,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:13" ht="60" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1212,7 +1233,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:13" ht="75" x14ac:dyDescent="0.25">
       <c r="B5" s="1" t="s">
         <v>48</v>
       </c>
@@ -1247,7 +1268,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:13" ht="60" x14ac:dyDescent="0.25">
       <c r="B6" s="1" t="s">
         <v>48</v>
       </c>
@@ -1285,7 +1306,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:13" ht="60" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
         <v>48</v>
       </c>
@@ -1320,7 +1341,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:13" ht="60" x14ac:dyDescent="0.25">
       <c r="B8" s="1" t="s">
         <v>48</v>
       </c>
@@ -1349,7 +1370,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="9" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:13" ht="60" x14ac:dyDescent="0.25">
       <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
@@ -1381,7 +1402,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:13" ht="75" x14ac:dyDescent="0.25">
       <c r="B10" s="1" t="s">
         <v>13</v>
       </c>
@@ -1410,7 +1431,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="11" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:13" ht="75" x14ac:dyDescent="0.25">
       <c r="B11" s="1" t="s">
         <v>48</v>
       </c>
@@ -1439,7 +1460,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="12" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:13" ht="60" x14ac:dyDescent="0.25">
       <c r="B12" s="1" t="s">
         <v>13</v>
       </c>
@@ -1468,7 +1489,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="13" spans="2:13" ht="72" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:13" ht="75" x14ac:dyDescent="0.25">
       <c r="B13" s="1" t="s">
         <v>13</v>
       </c>
@@ -1503,7 +1524,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="14" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:13" ht="60" x14ac:dyDescent="0.25">
       <c r="B14" s="1" t="s">
         <v>48</v>
       </c>
@@ -1532,7 +1553,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="15" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:13" ht="75" x14ac:dyDescent="0.25">
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1567,7 +1588,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="16" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:13" ht="30" x14ac:dyDescent="0.25">
       <c r="B16" s="1" t="s">
         <v>13</v>
       </c>
@@ -1590,7 +1611,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="17" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B17" s="1" t="s">
         <v>48</v>
       </c>
@@ -1619,7 +1640,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B18" s="1" t="s">
         <v>48</v>
       </c>
@@ -1648,7 +1669,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="19" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="19" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B19" s="1" t="s">
         <v>13</v>
       </c>
@@ -1673,8 +1694,11 @@
       <c r="I19" s="2" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="20" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="J19" s="1" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="20" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B20" s="1" t="s">
         <v>13</v>
       </c>
@@ -1699,8 +1723,11 @@
       <c r="I20" s="2" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="21" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="J20" s="1" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="21" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B21" s="1" t="s">
         <v>48</v>
       </c>
@@ -1725,8 +1752,11 @@
       <c r="I21" s="2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="22" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="J21" s="1" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="22" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B22" s="1" t="s">
         <v>48</v>
       </c>
@@ -1751,8 +1781,11 @@
       <c r="I22" s="2" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="23" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="J22" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="23" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B23" s="1" t="s">
         <v>48</v>
       </c>
@@ -1777,8 +1810,11 @@
       <c r="I23" s="2" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="24" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="J23" s="1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="24" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B24" s="1" t="s">
         <v>48</v>
       </c>
@@ -1803,8 +1839,11 @@
       <c r="I24" s="2" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="25" spans="2:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="J24" s="1" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="25" spans="2:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B25" s="1" t="s">
         <v>48</v>
       </c>
@@ -1829,8 +1868,11 @@
       <c r="I25" s="2" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="26" spans="2:10" ht="72" x14ac:dyDescent="0.3">
+      <c r="J25" s="1" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="26" spans="2:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B26" s="1" t="s">
         <v>48</v>
       </c>
@@ -1855,8 +1897,11 @@
       <c r="I26" s="2" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="27" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="J26" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="27" spans="2:10" ht="45" x14ac:dyDescent="0.25">
       <c r="B27" s="1" t="s">
         <v>48</v>
       </c>
@@ -1876,7 +1921,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="28" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="28" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>48</v>
       </c>
@@ -1902,7 +1947,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="29" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="29" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
         <v>48</v>
       </c>
@@ -1928,7 +1973,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="30" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="30" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
         <v>48</v>
       </c>
@@ -1954,7 +1999,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="31" spans="2:10" x14ac:dyDescent="0.3">
+    <row r="31" spans="2:10" ht="15" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>48</v>
       </c>
@@ -1974,7 +2019,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="32" spans="2:10" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
         <v>48</v>
       </c>
@@ -2000,7 +2045,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="33" spans="2:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="33" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
         <v>48</v>
       </c>
@@ -2026,7 +2071,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="34" spans="2:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="34" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
         <v>48</v>
       </c>
@@ -2052,7 +2097,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="35" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
+    <row r="35" spans="2:10" ht="105" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
         <v>48</v>
       </c>
@@ -2078,7 +2123,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="36" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="36" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
         <v>48</v>
       </c>
@@ -2104,7 +2149,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="2:10" ht="72" x14ac:dyDescent="0.3">
+    <row r="37" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
         <v>48</v>
       </c>
@@ -2130,7 +2175,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="38" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="38" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B38" s="1" t="s">
         <v>48</v>
       </c>
@@ -2159,7 +2204,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="39" spans="2:10" x14ac:dyDescent="0.3"/>
+    <row r="39" spans="2:10" ht="15" x14ac:dyDescent="0.25"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>

</xml_diff>

<commit_message>
to the small one!
</commit_message>
<xml_diff>
--- a/The Report/Requirements specification.xlsx
+++ b/The Report/Requirements specification.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Marvellous-Meal-Maker\The Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D836034-176A-46FE-BB7A-26FAACC66CEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A77F3E-B474-4C3F-8BD0-C168B0DE903E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="230">
   <si>
     <t>Requirement</t>
   </si>
@@ -632,10 +632,6 @@
     <t>Purchasing items will be required for certain methodologies, if not all, and as such outlining what the user needs to buy would help</t>
   </si>
   <si>
-    <t xml:space="preserve">Items can be purchased for methods
-</t>
-  </si>
-  <si>
     <t>Leftover factorisation for end products</t>
   </si>
   <si>
@@ -728,6 +724,39 @@
   </si>
   <si>
     <t>MethodBodge, items that are bodging for something else are noted in the pantry and what they become in the pantry, DeclareMethodBodge ChangeMethodBodge RemoveMethodBodge ListMethodsVariants</t>
+  </si>
+  <si>
+    <t>TheAlgorithm, store all component parts as floats to be able to randomly allocate out to the planner for allocation, ConnectToPlanner ConnectToMemory ConnectToPantry ConnectToRecipes GiveMeANewWeek</t>
+  </si>
+  <si>
+    <t>LogicPlanner, store potential products as str, DisplayCurrentWeeksPlan SaveWeekIntoSlot</t>
+  </si>
+  <si>
+    <t>StoreSettings, ingredients from certain stores as pantry items Allocations to specific types and kinds of stores as str Add bodgeness here too, AddStoreType RemoveStoreType LinkStoreToItem RemoveItemFromStore ListItemsStores ListStoresItems</t>
+  </si>
+  <si>
+    <t>AllergySettings, allergy to flag down noted in previous allergy sections and given a bool function here that you can toggle, AddUserAllergy RemoveUserAllergy TempAddUserAllergyForCertainTime</t>
+  </si>
+  <si>
+    <t>FourLoves, preferences stored as str with weights associated with them as floats of 0.5, 0.75, 1.25 and 1.5 respectively Allocate this to everything that needs it, AddItemPref ChangeItemPref RemoveItemPref AddMethodPref ChangeMethodPref RemoveMethodPref Add/Change/RemoveCuisinePref</t>
+  </si>
+  <si>
+    <t>Items can be purchased for methods</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MealtimeSlots, names as str Times set as float Tie into the Planner, DeclareTimeSlot RemoveTimeSlot </t>
+  </si>
+  <si>
+    <t>7DaysMem, memory weight modifiers as float Days named as str, Create7 (then allocate and call to it)</t>
+  </si>
+  <si>
+    <t>28DaysMem, memory weight modifiers as float Days named as str, Create28 (then allocate and call to it)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factoring, having the meal be factored will be a bool, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">WeeklyList, , </t>
   </si>
 </sst>
 </file>
@@ -1163,7 +1192,7 @@
         <v>6</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>120</v>
@@ -1189,7 +1218,7 @@
         <v>53</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="L3" s="1" t="s">
         <v>9</v>
@@ -1224,7 +1253,7 @@
         <v>52</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="L4" s="1" t="s">
         <v>5</v>
@@ -1250,7 +1279,7 @@
         <v>50</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>93</v>
@@ -1259,7 +1288,7 @@
         <v>51</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="L5" s="1" t="s">
         <v>13</v>
@@ -1294,10 +1323,10 @@
         <v>54</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="L6" s="1" t="s">
         <v>14</v>
@@ -1332,7 +1361,7 @@
         <v>55</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>48</v>
@@ -1367,7 +1396,7 @@
         <v>56</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="9" spans="2:13" ht="60" x14ac:dyDescent="0.25">
@@ -1396,7 +1425,7 @@
         <v>57</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="M9" s="1" t="s">
         <v>94</v>
@@ -1428,7 +1457,7 @@
         <v>58</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="11" spans="2:13" ht="75" x14ac:dyDescent="0.25">
@@ -1457,7 +1486,7 @@
         <v>59</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="12" spans="2:13" ht="60" x14ac:dyDescent="0.25">
@@ -1486,7 +1515,7 @@
         <v>60</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="13" spans="2:13" ht="75" x14ac:dyDescent="0.25">
@@ -1515,7 +1544,7 @@
         <v>61</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="K13" s="1" t="s">
         <v>116</v>
@@ -1550,7 +1579,7 @@
         <v>62</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="15" spans="2:13" ht="75" x14ac:dyDescent="0.25">
@@ -1579,7 +1608,7 @@
         <v>63</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K15" s="1" t="s">
         <v>122</v>
@@ -1608,7 +1637,7 @@
         <v>53</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="17" spans="2:10" ht="75" x14ac:dyDescent="0.25">
@@ -1637,7 +1666,7 @@
         <v>64</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="18" spans="2:10" ht="90" x14ac:dyDescent="0.25">
@@ -1666,7 +1695,7 @@
         <v>65</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="19" spans="2:10" ht="60" x14ac:dyDescent="0.25">
@@ -1695,7 +1724,7 @@
         <v>66</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="20" spans="2:10" ht="60" x14ac:dyDescent="0.25">
@@ -1724,7 +1753,7 @@
         <v>67</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="21" spans="2:10" ht="60" x14ac:dyDescent="0.25">
@@ -1753,7 +1782,7 @@
         <v>68</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="22" spans="2:10" ht="60" x14ac:dyDescent="0.25">
@@ -1782,7 +1811,7 @@
         <v>69</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="23" spans="2:10" ht="75" x14ac:dyDescent="0.25">
@@ -1811,7 +1840,7 @@
         <v>74</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="24" spans="2:10" ht="60" x14ac:dyDescent="0.25">
@@ -1840,7 +1869,7 @@
         <v>75</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="25" spans="2:10" ht="90" x14ac:dyDescent="0.25">
@@ -1869,7 +1898,7 @@
         <v>76</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="26" spans="2:10" ht="90" x14ac:dyDescent="0.25">
@@ -1889,7 +1918,7 @@
         <v>50</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>164</v>
@@ -1898,7 +1927,7 @@
         <v>77</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="27" spans="2:10" ht="45" x14ac:dyDescent="0.25">
@@ -1920,8 +1949,11 @@
       <c r="I27" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="28" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="J27" s="1" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="28" spans="2:10" ht="90" x14ac:dyDescent="0.25">
       <c r="B28" s="1" t="s">
         <v>48</v>
       </c>
@@ -1946,6 +1978,9 @@
       <c r="I28" s="2" t="s">
         <v>78</v>
       </c>
+      <c r="J28" s="1" t="s">
+        <v>221</v>
+      </c>
     </row>
     <row r="29" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B29" s="1" t="s">
@@ -1972,8 +2007,11 @@
       <c r="I29" s="2" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="30" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="J29" s="1" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="30" spans="2:10" ht="105" x14ac:dyDescent="0.25">
       <c r="B30" s="1" t="s">
         <v>48</v>
       </c>
@@ -1998,8 +2036,11 @@
       <c r="I30" s="2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="31" spans="2:10" ht="15" x14ac:dyDescent="0.25">
+      <c r="J30" s="1" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="31" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B31" s="1" t="s">
         <v>48</v>
       </c>
@@ -2018,8 +2059,11 @@
       <c r="I31" s="1" t="s">
         <v>53</v>
       </c>
-    </row>
-    <row r="32" spans="2:10" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="J31" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="32" spans="2:10" ht="60" x14ac:dyDescent="0.25">
       <c r="B32" s="1" t="s">
         <v>48</v>
       </c>
@@ -2044,6 +2088,9 @@
       <c r="I32" s="2" t="s">
         <v>81</v>
       </c>
+      <c r="J32" s="1" t="s">
+        <v>225</v>
+      </c>
     </row>
     <row r="33" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B33" s="1" t="s">
@@ -2070,6 +2117,9 @@
       <c r="I33" s="2" t="s">
         <v>82</v>
       </c>
+      <c r="J33" s="1" t="s">
+        <v>226</v>
+      </c>
     </row>
     <row r="34" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B34" s="1" t="s">
@@ -2096,6 +2146,9 @@
       <c r="I34" s="2" t="s">
         <v>83</v>
       </c>
+      <c r="J34" s="1" t="s">
+        <v>227</v>
+      </c>
     </row>
     <row r="35" spans="2:10" ht="105" x14ac:dyDescent="0.25">
       <c r="B35" s="1" t="s">
@@ -2122,6 +2175,9 @@
       <c r="I35" s="2" t="s">
         <v>84</v>
       </c>
+      <c r="J35" s="1" t="s">
+        <v>228</v>
+      </c>
     </row>
     <row r="36" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B36" s="1" t="s">
@@ -2143,11 +2199,14 @@
         <v>187</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>188</v>
+        <v>224</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>85</v>
       </c>
+      <c r="J36" s="1" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="37" spans="2:10" ht="75" x14ac:dyDescent="0.25">
       <c r="B37" s="1" t="s">
@@ -2160,16 +2219,16 @@
         <v>44</v>
       </c>
       <c r="E37" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="G37" s="1" t="s">
         <v>189</v>
       </c>
-      <c r="F37" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="G37" s="1" t="s">
+      <c r="H37" s="1" t="s">
         <v>190</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>191</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>86</v>
@@ -2201,7 +2260,7 @@
         <v>87</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="39" spans="2:10" ht="15" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
An entry in the futa
</commit_message>
<xml_diff>
--- a/The Report/Requirements specification.xlsx
+++ b/The Report/Requirements specification.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Marvellous-Meal-Maker\The Report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kidic\Documents\Computer Science\Project Work\The Report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A77F3E-B474-4C3F-8BD0-C168B0DE903E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECFEBDB4-2343-45B8-9586-BA20A6A1BECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="231">
   <si>
     <t>Requirement</t>
   </si>
@@ -753,10 +753,13 @@
     <t>28DaysMem, memory weight modifiers as float Days named as str, Create28 (then allocate and call to it)</t>
   </si>
   <si>
-    <t xml:space="preserve">Factoring, having the meal be factored will be a bool, </t>
-  </si>
-  <si>
-    <t xml:space="preserve">WeeklyList, , </t>
+    <t>Factoring, having the meal be factored will be a bool If the new meal is a recipe we should be able to add it to the list, TargetMealSlotIsOccupied</t>
+  </si>
+  <si>
+    <t>WeeklyExpirations, copy data from for methods we just want to put it in a way that the algorithmn can reslot the food if leftovers exist, TargetMealHasLeftovers</t>
+  </si>
+  <si>
+    <t>WeeklyList, this is to make the algorithm know where the stores are because up to this point it doesn't know what to do with the information, StoreForAlgorithm</t>
   </si>
 </sst>
 </file>
@@ -1149,24 +1152,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:M39"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="14.45" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="1"/>
-    <col min="2" max="2" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="14.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="29.7109375" style="1" customWidth="1"/>
-    <col min="8" max="8" width="24.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="49.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="47.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="15.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.5703125" style="1" customWidth="1"/>
-    <col min="13" max="16384" width="8.85546875" style="1"/>
+    <col min="4" max="4" width="31.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="29.6640625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="24.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="49.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="47.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.5546875" style="1" customWidth="1"/>
+    <col min="13" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:13" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1198,7 +1201,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="2:13" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>48</v>
       </c>
@@ -1227,7 +1230,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1262,7 +1265,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="2:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>48</v>
       </c>
@@ -1297,7 +1300,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>48</v>
       </c>
@@ -1335,7 +1338,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>48</v>
       </c>
@@ -1370,7 +1373,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:13" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B8" s="1" t="s">
         <v>48</v>
       </c>
@@ -1399,7 +1402,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="9" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>48</v>
       </c>
@@ -1431,7 +1434,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="10" spans="2:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>13</v>
       </c>
@@ -1460,7 +1463,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="11" spans="2:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>48</v>
       </c>
@@ -1489,7 +1492,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="12" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>13</v>
       </c>
@@ -1518,7 +1521,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="13" spans="2:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:13" ht="72" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>13</v>
       </c>
@@ -1553,7 +1556,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="14" spans="2:13" ht="60" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>48</v>
       </c>
@@ -1582,7 +1585,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="2:13" ht="75" x14ac:dyDescent="0.25">
+    <row r="15" spans="2:13" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1617,7 +1620,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="16" spans="2:13" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="2:13" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>13</v>
       </c>
@@ -1640,7 +1643,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="17" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>48</v>
       </c>
@@ -1669,7 +1672,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="18" spans="2:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
         <v>48</v>
       </c>
@@ -1698,7 +1701,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="19" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
         <v>13</v>
       </c>
@@ -1727,7 +1730,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="20" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B20" s="1" t="s">
         <v>13</v>
       </c>
@@ -1756,7 +1759,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="21" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:10" ht="43.2" x14ac:dyDescent="0.3">
       <c r="B21" s="1" t="s">
         <v>48</v>
       </c>
@@ -1785,7 +1788,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="22" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B22" s="1" t="s">
         <v>48</v>
       </c>
@@ -1814,7 +1817,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="23" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B23" s="1" t="s">
         <v>48</v>
       </c>
@@ -1843,7 +1846,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="24" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B24" s="1" t="s">
         <v>48</v>
       </c>
@@ -1872,7 +1875,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="25" spans="2:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B25" s="1" t="s">
         <v>48</v>
       </c>
@@ -1901,7 +1904,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="26" spans="2:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B26" s="1" t="s">
         <v>48</v>
       </c>
@@ -1930,7 +1933,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="27" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:10" ht="28.8" x14ac:dyDescent="0.3">
       <c r="B27" s="1" t="s">
         <v>48</v>
       </c>
@@ -1953,7 +1956,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="28" spans="2:10" ht="90" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B28" s="1" t="s">
         <v>48</v>
       </c>
@@ -1982,7 +1985,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="29" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B29" s="1" t="s">
         <v>48</v>
       </c>
@@ -2011,7 +2014,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="30" spans="2:10" ht="105" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B30" s="1" t="s">
         <v>48</v>
       </c>
@@ -2040,7 +2043,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="31" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B31" s="1" t="s">
         <v>48</v>
       </c>
@@ -2063,7 +2066,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="32" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B32" s="1" t="s">
         <v>48</v>
       </c>
@@ -2092,7 +2095,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="33" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B33" s="1" t="s">
         <v>48</v>
       </c>
@@ -2121,7 +2124,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="34" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B34" s="1" t="s">
         <v>48</v>
       </c>
@@ -2150,7 +2153,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="35" spans="2:10" ht="105" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:10" ht="86.4" x14ac:dyDescent="0.3">
       <c r="B35" s="1" t="s">
         <v>48</v>
       </c>
@@ -2179,7 +2182,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="36" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B36" s="1" t="s">
         <v>48</v>
       </c>
@@ -2205,10 +2208,10 @@
         <v>85</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="37" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="37" spans="2:10" ht="72" x14ac:dyDescent="0.3">
       <c r="B37" s="1" t="s">
         <v>48</v>
       </c>
@@ -2233,8 +2236,11 @@
       <c r="I37" s="2" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="38" spans="2:10" ht="60" x14ac:dyDescent="0.25">
+      <c r="J37" s="1" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="38" spans="2:10" ht="57.6" x14ac:dyDescent="0.3">
       <c r="B38" s="1" t="s">
         <v>48</v>
       </c>
@@ -2263,7 +2269,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="39" spans="2:10" ht="15" x14ac:dyDescent="0.25"/>
+    <row r="39" spans="2:10" x14ac:dyDescent="0.3"/>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <hyperlinks>

</xml_diff>